<commit_message>
Actualización e implementación de las funciones en utilerías, PDF de documentación del proyecto
</commit_message>
<xml_diff>
--- a/proyectosModuloII/SistemaEnrutamientoTiendasAutoservicio/MaterialesDeReferencia/datos_distribucion_tiendas.xlsx
+++ b/proyectosModuloII/SistemaEnrutamientoTiendasAutoservicio/MaterialesDeReferencia/datos_distribucion_tiendas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29912"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ZM\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1113ac1d89dbb239/Drive/Tec/VSC-workspace/Git_VSC/Git-TopicosIA/Git-TopicosIA/proyectosModuloII/SistemaEnrutamientoTiendasAutoservicio/MaterialesDeReferencia/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5BEA315-6D75-4FAA-845E-B8A7393F1117}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="348" yWindow="216" windowWidth="13764" windowHeight="11736" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -381,7 +381,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -743,18 +743,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G101"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -777,7 +777,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -800,7 +800,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -823,7 +823,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -846,7 +846,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -869,7 +869,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -892,7 +892,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -915,7 +915,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -938,7 +938,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -961,7 +961,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>7</v>
       </c>
@@ -984,7 +984,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -1007,7 +1007,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -1030,7 +1030,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -1053,7 +1053,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>19</v>
       </c>
@@ -1076,7 +1076,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -1099,7 +1099,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -1122,7 +1122,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>19</v>
       </c>
@@ -1145,7 +1145,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>19</v>
       </c>
@@ -1168,7 +1168,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>19</v>
       </c>
@@ -1191,7 +1191,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:7">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -1214,7 +1214,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:7">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -1237,7 +1237,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:7">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>19</v>
       </c>
@@ -1260,7 +1260,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:7">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>19</v>
       </c>
@@ -1283,7 +1283,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:7">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>19</v>
       </c>
@@ -1306,7 +1306,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="25" spans="1:7">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>19</v>
       </c>
@@ -1329,7 +1329,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="26" spans="1:7">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>19</v>
       </c>
@@ -1352,7 +1352,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="27" spans="1:7">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>19</v>
       </c>
@@ -1375,7 +1375,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:7">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>19</v>
       </c>
@@ -1398,7 +1398,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="1:7">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>19</v>
       </c>
@@ -1421,7 +1421,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="30" spans="1:7">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>19</v>
       </c>
@@ -1444,7 +1444,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="31" spans="1:7">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>19</v>
       </c>
@@ -1467,7 +1467,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="32" spans="1:7">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>19</v>
       </c>
@@ -1490,7 +1490,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="33" spans="1:7">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>19</v>
       </c>
@@ -1513,7 +1513,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="34" spans="1:7">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>19</v>
       </c>
@@ -1536,7 +1536,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="35" spans="1:7">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>19</v>
       </c>
@@ -1559,7 +1559,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="36" spans="1:7">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>19</v>
       </c>
@@ -1582,7 +1582,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="1:7">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>19</v>
       </c>
@@ -1605,7 +1605,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="38" spans="1:7">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>19</v>
       </c>
@@ -1628,7 +1628,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="39" spans="1:7">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>19</v>
       </c>
@@ -1651,7 +1651,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="40" spans="1:7">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>19</v>
       </c>
@@ -1674,7 +1674,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="41" spans="1:7">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>19</v>
       </c>
@@ -1697,7 +1697,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="42" spans="1:7">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>19</v>
       </c>
@@ -1720,7 +1720,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="43" spans="1:7">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>19</v>
       </c>
@@ -1743,7 +1743,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="44" spans="1:7">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>19</v>
       </c>
@@ -1766,7 +1766,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="45" spans="1:7">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>19</v>
       </c>
@@ -1789,7 +1789,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="46" spans="1:7">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>19</v>
       </c>
@@ -1812,7 +1812,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="47" spans="1:7">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>19</v>
       </c>
@@ -1835,7 +1835,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="48" spans="1:7">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>19</v>
       </c>
@@ -1858,7 +1858,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="49" spans="1:7">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>19</v>
       </c>
@@ -1881,7 +1881,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="50" spans="1:7">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>19</v>
       </c>
@@ -1904,7 +1904,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="51" spans="1:7">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>19</v>
       </c>
@@ -1927,7 +1927,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="52" spans="1:7">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>19</v>
       </c>
@@ -1950,7 +1950,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="53" spans="1:7">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>19</v>
       </c>
@@ -1973,7 +1973,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="54" spans="1:7">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>19</v>
       </c>
@@ -1996,7 +1996,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="55" spans="1:7">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>19</v>
       </c>
@@ -2019,7 +2019,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="56" spans="1:7">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>19</v>
       </c>
@@ -2042,7 +2042,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="57" spans="1:7">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>19</v>
       </c>
@@ -2065,7 +2065,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="58" spans="1:7">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>19</v>
       </c>
@@ -2088,7 +2088,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="59" spans="1:7">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>19</v>
       </c>
@@ -2111,7 +2111,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="60" spans="1:7">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>19</v>
       </c>
@@ -2134,7 +2134,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="61" spans="1:7">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>19</v>
       </c>
@@ -2157,7 +2157,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="62" spans="1:7">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>19</v>
       </c>
@@ -2180,7 +2180,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="63" spans="1:7">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>19</v>
       </c>
@@ -2203,7 +2203,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="64" spans="1:7">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>19</v>
       </c>
@@ -2226,7 +2226,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="65" spans="1:7">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>19</v>
       </c>
@@ -2249,7 +2249,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="66" spans="1:7">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>19</v>
       </c>
@@ -2272,7 +2272,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="67" spans="1:7">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>19</v>
       </c>
@@ -2295,7 +2295,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="68" spans="1:7">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>19</v>
       </c>
@@ -2318,7 +2318,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="69" spans="1:7">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>19</v>
       </c>
@@ -2341,7 +2341,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="70" spans="1:7">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>19</v>
       </c>
@@ -2364,7 +2364,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="71" spans="1:7">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>19</v>
       </c>
@@ -2387,7 +2387,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="72" spans="1:7">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>19</v>
       </c>
@@ -2410,7 +2410,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="73" spans="1:7">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>19</v>
       </c>
@@ -2433,7 +2433,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="74" spans="1:7">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>19</v>
       </c>
@@ -2456,7 +2456,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="75" spans="1:7">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>19</v>
       </c>
@@ -2479,7 +2479,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="76" spans="1:7">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>19</v>
       </c>
@@ -2502,7 +2502,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="77" spans="1:7">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>19</v>
       </c>
@@ -2525,7 +2525,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="78" spans="1:7">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>19</v>
       </c>
@@ -2548,7 +2548,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="79" spans="1:7">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>19</v>
       </c>
@@ -2571,7 +2571,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="80" spans="1:7">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>19</v>
       </c>
@@ -2594,7 +2594,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="81" spans="1:7">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>19</v>
       </c>
@@ -2617,7 +2617,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="82" spans="1:7">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>19</v>
       </c>
@@ -2640,7 +2640,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="83" spans="1:7">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>19</v>
       </c>
@@ -2663,7 +2663,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="84" spans="1:7">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>19</v>
       </c>
@@ -2686,7 +2686,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="85" spans="1:7">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>19</v>
       </c>
@@ -2709,7 +2709,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="86" spans="1:7">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>19</v>
       </c>
@@ -2732,7 +2732,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="87" spans="1:7">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>19</v>
       </c>
@@ -2755,7 +2755,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="88" spans="1:7">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>19</v>
       </c>
@@ -2778,7 +2778,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="89" spans="1:7">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>19</v>
       </c>
@@ -2801,7 +2801,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="90" spans="1:7">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>19</v>
       </c>
@@ -2824,7 +2824,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="91" spans="1:7">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>19</v>
       </c>
@@ -2847,7 +2847,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="92" spans="1:7">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>19</v>
       </c>
@@ -2870,7 +2870,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="93" spans="1:7">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>19</v>
       </c>
@@ -2893,7 +2893,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="94" spans="1:7">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>19</v>
       </c>
@@ -2916,7 +2916,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="95" spans="1:7">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>19</v>
       </c>
@@ -2939,7 +2939,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="96" spans="1:7">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>19</v>
       </c>
@@ -2962,7 +2962,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="97" spans="1:7">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>19</v>
       </c>
@@ -2985,7 +2985,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="98" spans="1:7">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>19</v>
       </c>
@@ -3008,7 +3008,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="99" spans="1:7">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>19</v>
       </c>
@@ -3031,7 +3031,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="100" spans="1:7">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>19</v>
       </c>
@@ -3054,7 +3054,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="101" spans="1:7">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>19</v>
       </c>
@@ -3083,15 +3083,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101000A507043A2ACA54B8490C0503A7704E1" ma:contentTypeVersion="4" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="1eb2ca4be7e08a340c0fe608cb198fdb">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e0b6cee9-4e7c-4b3e-b288-e0d65ed205ae" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0327b537c0e2a22b7da7c84723604bd8" ns2:_="">
     <xsd:import namespace="e0b6cee9-4e7c-4b3e-b288-e0d65ed205ae"/>
@@ -3235,6 +3226,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -3244,13 +3244,37 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B235EF15-1914-4E86-A3FC-C4AFF5D42EFE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{852AFE2A-4E31-4AF6-A823-4ED7D7D38EF9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="e0b6cee9-4e7c-4b3e-b288-e0d65ed205ae"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{852AFE2A-4E31-4AF6-A823-4ED7D7D38EF9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B235EF15-1914-4E86-A3FC-C4AFF5D42EFE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F4B49499-F952-4962-8962-ED8459477F70}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F4B49499-F952-4962-8962-ED8459477F70}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e0b6cee9-4e7c-4b3e-b288-e0d65ed205ae"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>